<commit_message>
change length to 59 closes #185
</commit_message>
<xml_diff>
--- a/data/epp-14-data.xlsx
+++ b/data/epp-14-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gavin.brown/Code/rst-test-specs/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5048BE27-AAC6-694A-BBD9-0720B2C6D77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C63246-FF93-1E4D-9467-22515B4282B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{CD472396-4CFB-9A45-AA99-46F4E9CB8B91}"/>
   </bookViews>
@@ -324,9 +324,6 @@
 * If the EPP server implements RFC 9154, then the `pw` field must be empty.</t>
   </si>
   <si>
-    <t>{"xn--" &amp; RANDASCII(60) &amp; "." &amp; $TLD}</t>
-  </si>
-  <si>
     <t>208.77.190.199</t>
   </si>
   <si>
@@ -362,6 +359,9 @@
   </si>
   <si>
     <t>keyData</t>
+  </si>
+  <si>
+    <t>{"xn--" &amp; RANDASCII(59) &amp; "." &amp; $TLD}</t>
   </si>
 </sst>
 </file>
@@ -1474,7 +1474,7 @@
     </row>
     <row r="5" spans="2:31" ht="128" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -1562,7 +1562,7 @@
         <v>36</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>52</v>
@@ -1631,7 +1631,7 @@
         <v>33</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>60</v>
@@ -1819,7 +1819,7 @@
     </row>
     <row r="12" spans="2:31" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="W12" s="1" t="s">
         <v>1</v>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="22" spans="3:24" x14ac:dyDescent="0.2">
       <c r="I22" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="W22" s="1" t="s">
         <v>2</v>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="23" spans="3:24" x14ac:dyDescent="0.2">
       <c r="I23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="W23" s="1" t="s">
         <v>1</v>
@@ -1972,7 +1972,7 @@
     </row>
     <row r="24" spans="3:24" x14ac:dyDescent="0.2">
       <c r="I24" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="W24" s="1" t="s">
         <v>1</v>
@@ -2019,7 +2019,7 @@
         <v>34</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="W28" s="1" t="s">
         <v>2</v>
@@ -2030,7 +2030,7 @@
     </row>
     <row r="29" spans="3:24" x14ac:dyDescent="0.2">
       <c r="J29" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="W29" s="1" t="s">
         <v>1</v>
@@ -2088,7 +2088,7 @@
         <v>34</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>34</v>
@@ -2210,7 +2210,7 @@
     </row>
     <row r="44" spans="8:24" x14ac:dyDescent="0.2">
       <c r="N44" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="R44" s="1" t="s">
         <v>80</v>

</xml_diff>